<commit_message>
Updated market place search plan reports
</commit_message>
<xml_diff>
--- a/data/marketplace/MarketplaceData.xlsx
+++ b/data/marketplace/MarketplaceData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molinahealthcare-my.sharepoint.com/personal/naresh_jangid_molinahealthcare_com/Documents/Automation/molina_automation/PlanMaterialAutomation/data/marketplace/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_5625D102A8BF400918838D571C15BBF580A02A0F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9CB97DC1-37DD-4E2F-9A90-81F054823C70}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_5625D102A8BF400918838D571C15BBF580A02A0F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{48662BB8-5DB8-4DE3-9730-2ADE31870552}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -686,9 +686,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -714,7 +714,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -740,7 +740,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -766,7 +766,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>17</v>
       </c>
@@ -792,7 +792,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -818,7 +818,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -844,7 +844,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -870,7 +870,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>17</v>
       </c>
@@ -896,7 +896,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -922,7 +922,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -948,7 +948,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -974,7 +974,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -1000,7 +1000,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -1026,7 +1026,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>17</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>17</v>
       </c>
@@ -1078,7 +1078,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -1104,7 +1104,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -1156,7 +1156,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1182,7 +1182,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>17</v>
       </c>
@@ -1245,12 +1245,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:J10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="31.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1282,9 +1282,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B2" t="s">
         <v>69</v>
@@ -1314,7 +1314,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1346,9 +1346,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
         <v>78</v>
@@ -1378,9 +1378,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
         <v>81</v>
@@ -1410,9 +1410,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
         <v>84</v>
@@ -1442,9 +1442,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
         <v>86</v>
@@ -1474,9 +1474,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
         <v>88</v>
@@ -1506,9 +1506,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
         <v>91</v>
@@ -1538,9 +1538,9 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
         <v>94</v>
@@ -1573,7 +1573,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:J10" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J1 A3:J3 B2:J2 B5:J10 B4:J4" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{5e625f8d-0b53-4f56-9e46-19fa14bb2e5c}" enabled="0" method="" siteId="{5e625f8d-0b53-4f56-9e46-19fa14bb2e5c}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>